<commit_message>
Add table board zone and guide page
</commit_message>
<xml_diff>
--- a/doc/愛我家鄉_開發指令工作簿.xlsx
+++ b/doc/愛我家鄉_開發指令工作簿.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="開發指令總覽" sheetId="1" r:id="R707be1a8a5fc4d65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="設計決策" sheetId="2" r:id="R363b2c46f65b4d4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="備份清單" sheetId="3" r:id="Rcd419db64bc64af1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="卡牌與系統" sheetId="4" r:id="R0fa94eb086d24973"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="開發指令總覽" sheetId="1" r:id="Rd2295fe3c9274b56"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="設計決策" sheetId="2" r:id="R89bb5710894044a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="備份清單" sheetId="3" r:id="R78067144aaa84bc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="卡牌與系統" sheetId="4" r:id="Rcd43d4beb95646df"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -335,7 +335,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="4" t="str">
-        <x:v>本工作簿記錄從原型、玩家視窗、圖資、HUD、AI、結局分析到本輪手牌整理放大與 GitHub 上傳的主要開發指令。</x:v>
+        <x:v>本工作簿記錄從原型、玩家視窗、圖資、HUD、AI、結局分析到本輪桌牌區獨立、說明頁、QR 與 GitHub Pages 公開啟用的主要開發指令。</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1305,6 +1305,23 @@
       </x:c>
       <x:c r="E60" s="10" t="str">
         <x:v>新增 hand-manage-overlay 中央手牌整理區；手牌夾與整理換牌按鈕可開啟放大面板，玩家回合可棄牌並補牌；完成語法與 smoke test，準備 GitHub 上傳。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="10" t="str">
+        <x:v>057</x:v>
+      </x:c>
+      <x:c r="B61" s="10" t="str">
+        <x:v>桌牌區獨立、說明頁與 GitHub Pages</x:v>
+      </x:c>
+      <x:c r="C61" s="10" t="str">
+        <x:v>將桌牌放置區命名為桌牌區並獨立程式；點擊桌牌區攻擊/防禦/加成可放大整理並棄牌換牌；小人每回合結束回中心、放牌後再出發；回到開局設定改成結束遊戲；首頁新增說明頁、小咪老師、QR Code；公開 GitHub 並啟用遊戲首頁。</x:v>
+      </x:c>
+      <x:c r="D61" s="10" t="str">
+        <x:v>完成</x:v>
+      </x:c>
+      <x:c r="E61" s="10" t="str">
+        <x:v>新增 table-board-zone.js；玩家視窗接上 table-board-overlay 與人流中心集合節奏；index 新增卡牌說明頁、感謝共同開發者、小咪老師解說與訂閱 QR；結局與感謝幕加入 QR；完成備份與工作簿更新。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1679,6 +1696,14 @@
         <x:v>D:/Codex/home_community_battle/workbook/backups/2026-06-17_before-targeted-attack</x:v>
       </x:c>
     </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="10" t="str">
+        <x:v>2026-06-18_before_table_board_zone_guide</x:v>
+      </x:c>
+      <x:c r="B33" s="10" t="str">
+        <x:v>D:/Codex/home_community_battle/workbook/backups/2026-06-18_before_table_board_zone_guide</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:B1"/>
@@ -1805,13 +1830,13 @@
         <x:v>本輪新增</x:v>
       </x:c>
       <x:c r="B10" s="10" t="str">
-        <x:v>手牌整理放大與換牌</x:v>
+        <x:v>桌牌區與說明頁</x:v>
       </x:c>
       <x:c r="C10" s="10" t="str">
-        <x:v>player_window/player-window.html</x:v>
+        <x:v>player_window/table-board-zone.js、player_window/player-window.html、index.html</x:v>
       </x:c>
       <x:c r="D10" s="10" t="str">
-        <x:v>點擊手牌夾或整理換牌可開啟中央手牌整理區，玩家回合可棄牌並補牌，避免被攻擊後卡住。</x:v>
+        <x:v>桌牌區命名並獨立模組；桌牌區可放大整理與棄置換牌；首頁說明頁展示攻防對照、主題卡、加成卡、小咪老師與訂閱 QR。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Add sponsor collaborator credits
</commit_message>
<xml_diff>
--- a/doc/愛我家鄉_開發指令工作簿.xlsx
+++ b/doc/愛我家鄉_開發指令工作簿.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="開發指令總覽" sheetId="1" r:id="Rd2295fe3c9274b56"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="設計決策" sheetId="2" r:id="R89bb5710894044a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="備份清單" sheetId="3" r:id="R78067144aaa84bc8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="卡牌與系統" sheetId="4" r:id="Rcd43d4beb95646df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="開發指令總覽" sheetId="1" r:id="R47f8b62f278947e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="設計決策" sheetId="2" r:id="R447435b59ab247fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="備份清單" sheetId="3" r:id="R1194116cf0224720"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="卡牌與系統" sheetId="4" r:id="Rc1aa9d823bfa4f06"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -335,7 +335,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="4" t="str">
-        <x:v>本工作簿記錄從原型、玩家視窗、圖資、HUD、AI、結局分析到本輪桌牌區獨立、說明頁、QR 與 GitHub Pages 公開啟用的主要開發指令。</x:v>
+        <x:v>本工作簿記錄從原型、玩家視窗、圖資、HUD、AI、結局分析到本輪贊助共同創作者名單掛載的主要開發指令。</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1322,6 +1322,23 @@
       </x:c>
       <x:c r="E61" s="10" t="str">
         <x:v>新增 table-board-zone.js；玩家視窗接上 table-board-overlay 與人流中心集合節奏；index 新增卡牌說明頁、感謝共同開發者、小咪老師解說與訂閱 QR；結局與感謝幕加入 QR；完成備份與工作簿更新。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="10" t="str">
+        <x:v>058</x:v>
+      </x:c>
+      <x:c r="B62" s="10" t="str">
+        <x:v>贊助共同創作者名單</x:v>
+      </x:c>
+      <x:c r="C62" s="10" t="str">
+        <x:v>把贊助共同創作者名單掛上去：林慶泓、陳連域、Bobo Chen、Tsai Kurt、Chungwei Hsieh、許士彥、林以泓、黃安志、孔祥宇、Ian Chen、潘慧君、陳民峰、Lili Lin、陳小葉、李仁耀、李英如、蔡昌樺、陳孝魁、陳慶源、傅欽杰。</x:v>
+      </x:c>
+      <x:c r="D62" s="10" t="str">
+        <x:v>完成</x:v>
+      </x:c>
+      <x:c r="E62" s="10" t="str">
+        <x:v>首頁說明頁新增贊助共同創作者名單網格；遊戲結束電影感謝幕新增贊助共同創作者專區。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1839,6 +1856,20 @@
         <x:v>桌牌區命名並獨立模組；桌牌區可放大整理與棄置換牌；首頁說明頁展示攻防對照、主題卡、加成卡、小咪老師與訂閱 QR。</x:v>
       </x:c>
     </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="10" t="str">
+        <x:v>本輪新增</x:v>
+      </x:c>
+      <x:c r="B11" s="10" t="str">
+        <x:v>贊助共同創作者名單</x:v>
+      </x:c>
+      <x:c r="C11" s="10" t="str">
+        <x:v>index.html、player_window/player-window.html</x:v>
+      </x:c>
+      <x:c r="D11" s="10" t="str">
+        <x:v>首頁說明頁與遊戲片尾感謝幕加入 20 位贊助共同創作者名單。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>

</xml_diff>

<commit_message>
Add teaching documents and manuals
</commit_message>
<xml_diff>
--- a/doc/愛我家鄉_開發指令工作簿.xlsx
+++ b/doc/愛我家鄉_開發指令工作簿.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="開發指令總覽" sheetId="1" r:id="R47f8b62f278947e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="設計決策" sheetId="2" r:id="R447435b59ab247fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="備份清單" sheetId="3" r:id="R1194116cf0224720"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="卡牌與系統" sheetId="4" r:id="Rc1aa9d823bfa4f06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="開發指令總覽" sheetId="1" r:id="R42393735d5184b14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="設計決策" sheetId="2" r:id="R45a93ce6058d4651"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="備份清單" sheetId="3" r:id="Rb845a7ac17964172"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="卡牌與系統" sheetId="4" r:id="R3f4fbb9358fa48f6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -335,7 +335,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="4" t="str">
-        <x:v>本工作簿記錄從原型、玩家視窗、圖資、HUD、AI、結局分析到本輪贊助共同創作者名單掛載的主要開發指令。</x:v>
+        <x:v>本工作簿記錄從原型、玩家視窗、圖資、HUD、AI、結局分析到本輪 108 課綱教案、玩家手冊與教師教學指引輸出的主要開發指令。</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1339,6 +1339,23 @@
       </x:c>
       <x:c r="E62" s="10" t="str">
         <x:v>首頁說明頁新增贊助共同創作者名單網格；遊戲結束電影感謝幕新增贊助共同創作者專區。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="10" t="str">
+        <x:v>059</x:v>
+      </x:c>
+      <x:c r="B63" s="10" t="str">
+        <x:v>教案、玩家手冊與教師指引</x:v>
+      </x:c>
+      <x:c r="C63" s="10" t="str">
+        <x:v>設計教學教案，要符合 108 課綱模式教案；另外是玩家操作手冊，寫給小學生看的；教學指引也寫一下；做成 doc 和 pdf 檔，另存在 doc 資料夾。</x:v>
+      </x:c>
+      <x:c r="D63" s="10" t="str">
+        <x:v>完成</x:v>
+      </x:c>
+      <x:c r="E63" s="10" t="str">
+        <x:v>新增三份文件：108 課綱模式教案、小學生玩家操作手冊、教師教學指引；各自輸出 DOCX 與 PDF，並加入文件生成腳本與 PDF 生成腳本。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1870,6 +1887,20 @@
         <x:v>首頁說明頁與遊戲片尾感謝幕加入 20 位贊助共同創作者名單。</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="10" t="str">
+        <x:v>本輪新增</x:v>
+      </x:c>
+      <x:c r="B12" s="10" t="str">
+        <x:v>教學文件</x:v>
+      </x:c>
+      <x:c r="C12" s="10" t="str">
+        <x:v>doc/*.docx、doc/*.pdf、doc/tools/build-teaching-docs.py、doc/tools/build-teaching-pdfs.py</x:v>
+      </x:c>
+      <x:c r="D12" s="10" t="str">
+        <x:v>新增 108 課綱模式教案、小學生玩家操作手冊、教師教學指引，並各自輸出 DOCX 與 PDF。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D1"/>

</xml_diff>

<commit_message>
Add trap slots and exchange limits
</commit_message>
<xml_diff>
--- a/doc/愛我家鄉_開發指令工作簿.xlsx
+++ b/doc/愛我家鄉_開發指令工作簿.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="開發指令總覽" sheetId="1" r:id="R42393735d5184b14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="設計決策" sheetId="2" r:id="R45a93ce6058d4651"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="備份清單" sheetId="3" r:id="Rb845a7ac17964172"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="卡牌與系統" sheetId="4" r:id="R3f4fbb9358fa48f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="開發指令總覽" sheetId="1" r:id="Rd2cc2e0c49924df6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="設計決策" sheetId="2" r:id="R69fcb750d68d49e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="備份清單" sheetId="3" r:id="Rf91ce3439f504440"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="卡牌與系統" sheetId="4" r:id="Rea233eb5db71423e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1358,6 +1358,23 @@
         <x:v>新增三份文件：108 課綱模式教案、小學生玩家操作手冊、教師教學指引；各自輸出 DOCX 與 PDF，並加入文件生成腳本與 PDF 生成腳本。</x:v>
       </x:c>
     </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="10" t="str">
+        <x:v>060</x:v>
+      </x:c>
+      <x:c r="B64" s="10" t="str">
+        <x:v>陷阱卡槽、商店與換牌限制</x:v>
+      </x:c>
+      <x:c r="C64" s="10" t="str">
+        <x:v>少了陷阱卡卡牌夾；桌牌區要多兩張陷阱卡對應並再拉大；陷阱卡可直接抵觸攻擊卡；換牌機制一回合只能換三張，出完手牌才刷手牌，不可棄牌馬上補；商店要買得到陷阱卡與防禦卡。</x:v>
+      </x:c>
+      <x:c r="D64" s="10" t="str">
+        <x:v>完成</x:v>
+      </x:c>
+      <x:c r="E64" s="10" t="str">
+        <x:v>桌牌區改成 3 攻、2 防、2 加成、2 陷阱；陷阱觸發後抵銷攻擊並進墳場；商店保證納入防禦/陷阱候選；手牌與桌牌整理換牌每回合最多 3 張，棄置不立即補牌，手牌打空或下回合開始才補滿。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:E1"/>
@@ -1738,6 +1755,14 @@
         <x:v>D:/Codex/home_community_battle/workbook/backups/2026-06-18_before_table_board_zone_guide</x:v>
       </x:c>
     </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="10" t="str">
+        <x:v>2026-06-18_before_trap_slots_shop_exchange_limit</x:v>
+      </x:c>
+      <x:c r="B34" s="10" t="str">
+        <x:v>D:/Codex/home_community_battle/workbook/backups/2026-06-18_before_trap_slots_shop_exchange_limit</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:B1"/>

</xml_diff>

<commit_message>
Animate crowd flow and HUD metrics
</commit_message>
<xml_diff>
--- a/doc/愛我家鄉_開發指令工作簿.xlsx
+++ b/doc/愛我家鄉_開發指令工作簿.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="開發指令總覽" sheetId="1" r:id="Rd2cc2e0c49924df6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="設計決策" sheetId="2" r:id="R69fcb750d68d49e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="備份清單" sheetId="3" r:id="Rf91ce3439f504440"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="卡牌與系統" sheetId="4" r:id="Rea233eb5db71423e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="開發指令總覽" sheetId="1" r:id="R48c08300da934d59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="設計決策" sheetId="2" r:id="R9555fcb688fc4ec9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="備份清單" sheetId="3" r:id="Rb9d48959925e4c4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="卡牌與系統" sheetId="4" r:id="R034a396de0f84450"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1375,6 +1375,23 @@
         <x:v>桌牌區改成 3 攻、2 防、2 加成、2 陷阱；陷阱觸發後抵銷攻擊並進墳場；商店保證納入防禦/陷阱候選；手牌與桌牌整理換牌每回合最多 3 張，棄置不立即補牌，手牌打空或下回合開始才補滿。</x:v>
       </x:c>
     </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="10" t="str">
+        <x:v>061</x:v>
+      </x:c>
+      <x:c r="B65" s="10" t="str">
+        <x:v>人流動畫與玩家指標直條圖</x:v>
+      </x:c>
+      <x:c r="C65" s="10" t="str">
+        <x:v>人流系統沒有動；玩家結束牌局後，小人與車輛要開始移動到各家；金流、滿意度、幸福度與人流要在玩家訊息中以直條圖呈現，每回合增減明顯，增加顯示 + 號，減少出現紅色警示。</x:v>
+      </x:c>
+      <x:c r="D65" s="10" t="str">
+        <x:v>完成</x:v>
+      </x:c>
+      <x:c r="E65" s="10" t="str">
+        <x:v>新增人流聚集中央後自動出發到四家的 departing 動畫；回合開始依主題、人流、民心與烏雲調整本月人潮；玩家 HUD 新增金流、資金、人潮、滿意度、幸福度直條圖與本回合正負增減提示，下降時顯示紅色警示。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:E1"/>
@@ -1749,17 +1766,25 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="10" t="str">
-        <x:v>2026-06-18_before_table_board_zone_guide</x:v>
+        <x:v>2026-06-18_before_crowd_flow_bars</x:v>
       </x:c>
       <x:c r="B33" s="10" t="str">
-        <x:v>D:/Codex/home_community_battle/workbook/backups/2026-06-18_before_table_board_zone_guide</x:v>
+        <x:v>D:/Codex/home_community_battle/workbook/backups/2026-06-18_before_crowd_flow_bars</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="10" t="str">
+        <x:v>2026-06-18_before_table_board_zone_guide</x:v>
+      </x:c>
+      <x:c r="B34" s="10" t="str">
+        <x:v>D:/Codex/home_community_battle/workbook/backups/2026-06-18_before_table_board_zone_guide</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="10" t="str">
         <x:v>2026-06-18_before_trap_slots_shop_exchange_limit</x:v>
       </x:c>
-      <x:c r="B34" s="10" t="str">
+      <x:c r="B35" s="10" t="str">
         <x:v>D:/Codex/home_community_battle/workbook/backups/2026-06-18_before_trap_slots_shop_exchange_limit</x:v>
       </x:c>
     </x:row>

</xml_diff>